<commit_message>
Update: addition of R7 & C8
</commit_message>
<xml_diff>
--- a/Data/sensor_locations_all_plots.xlsx
+++ b/Data/sensor_locations_all_plots.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ugentbe-my.sharepoint.com/personal/egvdwall_vandewalle_ugent_be/Documents/Documenten/PhD CAVElab/Code PhD/ForEdgeClimOnPanama/Data/Data_Kasper/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ugentbe-my.sharepoint.com/personal/egvdwall_vandewalle_ugent_be/Documents/Documenten/PhD CAVElab/Code PhD/ForEdgeClimOnPanama/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="8_{1F05EFE1-A1B1-46D8-97A0-A405852F5B9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96EF3346-2256-431D-9C12-5E731DDD54E3}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{1F05EFE1-A1B1-46D8-97A0-A405852F5B9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9831A3B6-C9E9-404C-8824-9D6CC08D086F}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sensor_locations" sheetId="1" r:id="rId1"/>
@@ -809,10 +809,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1112,11 +1108,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:H310"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1142,7 +1137,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1.95</v>
       </c>
@@ -1168,7 +1163,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>35.140999999999998</v>
       </c>
@@ -1194,7 +1189,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>56.088000000000001</v>
       </c>
@@ -1220,7 +1215,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>54.073</v>
       </c>
@@ -1246,7 +1241,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>20</v>
       </c>
@@ -1272,7 +1267,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6.6829999999999998</v>
       </c>
@@ -1298,7 +1293,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>15.321</v>
       </c>
@@ -1324,7 +1319,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>24.724</v>
       </c>
@@ -1350,7 +1345,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>54.27</v>
       </c>
@@ -1376,7 +1371,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>13.468</v>
       </c>
@@ -1402,7 +1397,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>21.666</v>
       </c>
@@ -1428,7 +1423,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>44.765999999999998</v>
       </c>
@@ -1454,7 +1449,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>56.256</v>
       </c>
@@ -1480,7 +1475,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>20.963999999999999</v>
       </c>
@@ -1506,7 +1501,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>5.4260000000000002</v>
       </c>
@@ -1532,7 +1527,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>19.431999999999999</v>
       </c>
@@ -1558,7 +1553,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>21.988</v>
       </c>
@@ -1584,7 +1579,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>47.298999999999999</v>
       </c>
@@ -1610,7 +1605,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>8.4830000000000005</v>
       </c>
@@ -1636,7 +1631,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>34.137</v>
       </c>
@@ -1662,7 +1657,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>55.482999999999997</v>
       </c>
@@ -1688,7 +1683,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>57.692999999999998</v>
       </c>
@@ -1714,7 +1709,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>37.164999999999999</v>
       </c>
@@ -1740,7 +1735,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>8.61</v>
       </c>
@@ -1766,7 +1761,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>13.42</v>
       </c>
@@ -1792,7 +1787,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>33.171999999999997</v>
       </c>
@@ -1818,7 +1813,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>57.64</v>
       </c>
@@ -1844,7 +1839,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>17.748999999999999</v>
       </c>
@@ -1870,7 +1865,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>34.792000000000002</v>
       </c>
@@ -1896,7 +1891,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>48.908999999999999</v>
       </c>
@@ -1922,7 +1917,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>49.356000000000002</v>
       </c>
@@ -1948,7 +1943,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>24.576000000000001</v>
       </c>
@@ -1974,7 +1969,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2.823</v>
       </c>
@@ -2000,7 +1995,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>0</v>
       </c>
@@ -2026,7 +2021,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>37.110999999999997</v>
       </c>
@@ -2052,7 +2047,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>44.527999999999999</v>
       </c>
@@ -2078,7 +2073,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>15.753</v>
       </c>
@@ -2104,7 +2099,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>22.414999999999999</v>
       </c>
@@ -2130,7 +2125,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>45.457000000000001</v>
       </c>
@@ -2156,7 +2151,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>48.42</v>
       </c>
@@ -2182,7 +2177,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>22.186</v>
       </c>
@@ -2208,7 +2203,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>14.065</v>
       </c>
@@ -2234,7 +2229,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>6.8129999999999997</v>
       </c>
@@ -2260,7 +2255,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>41.509</v>
       </c>
@@ -2286,7 +2281,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>50.892000000000003</v>
       </c>
@@ -2312,7 +2307,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>7.4610000000000003</v>
       </c>
@@ -2338,7 +2333,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>27.39</v>
       </c>
@@ -2364,7 +2359,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>56.170999999999999</v>
       </c>
@@ -2390,7 +2385,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>53.58</v>
       </c>
@@ -2416,7 +2411,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>21.745000000000001</v>
       </c>
@@ -2442,7 +2437,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>3.5379999999999998</v>
       </c>
@@ -2468,7 +2463,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>5.609</v>
       </c>
@@ -2494,7 +2489,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>32.768999999999998</v>
       </c>
@@ -2520,7 +2515,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>47.738</v>
       </c>
@@ -2546,7 +2541,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>1.28</v>
       </c>
@@ -2572,7 +2567,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>24.138999999999999</v>
       </c>
@@ -2598,7 +2593,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>48.341999999999999</v>
       </c>
@@ -2624,7 +2619,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>52.316000000000003</v>
       </c>
@@ -2650,7 +2645,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>31.856000000000002</v>
       </c>
@@ -2676,7 +2671,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>14.21</v>
       </c>
@@ -2702,7 +2697,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>13.057</v>
       </c>
@@ -2728,7 +2723,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>28.994</v>
       </c>
@@ -2754,7 +2749,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>41.862000000000002</v>
       </c>
@@ -2780,7 +2775,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>9.0030000000000001</v>
       </c>
@@ -2806,7 +2801,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>12.946999999999999</v>
       </c>
@@ -2832,7 +2827,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>19.628</v>
       </c>
@@ -2858,7 +2853,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>20</v>
       </c>
@@ -2878,7 +2873,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>23.338000000000001</v>
       </c>
@@ -2904,7 +2899,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>27.991</v>
       </c>
@@ -2930,7 +2925,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>46.073999999999998</v>
       </c>
@@ -2956,7 +2951,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>50.768000000000001</v>
       </c>
@@ -2982,7 +2977,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>22.052</v>
       </c>
@@ -3008,7 +3003,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>31.552</v>
       </c>
@@ -3034,7 +3029,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>31.302</v>
       </c>
@@ -3060,7 +3055,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>32.11</v>
       </c>
@@ -3086,7 +3081,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>29.347999999999999</v>
       </c>
@@ -3112,7 +3107,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="78" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>6.6150000000000002</v>
       </c>
@@ -3138,7 +3133,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>10.334</v>
       </c>
@@ -3164,7 +3159,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>11.755000000000001</v>
       </c>
@@ -3190,7 +3185,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>6.508</v>
       </c>
@@ -3216,7 +3211,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>4.7919999999999998</v>
       </c>
@@ -3242,7 +3237,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>11.646000000000001</v>
       </c>
@@ -3268,7 +3263,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>6.9729999999999999</v>
       </c>
@@ -3294,7 +3289,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>2.4249999999999998</v>
       </c>
@@ -3320,7 +3315,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>34.630000000000003</v>
       </c>
@@ -3346,7 +3341,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>51.707000000000001</v>
       </c>
@@ -3372,7 +3367,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>52.82</v>
       </c>
@@ -3398,7 +3393,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>55.820999999999998</v>
       </c>
@@ -3424,7 +3419,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>57.895000000000003</v>
       </c>
@@ -3450,7 +3445,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>43.244</v>
       </c>
@@ -3476,7 +3471,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>8.3810000000000002</v>
       </c>
@@ -3502,7 +3497,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>5.8650000000000002</v>
       </c>
@@ -3528,7 +3523,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>39.704999999999998</v>
       </c>
@@ -3554,7 +3549,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>51.826999999999998</v>
       </c>
@@ -3580,7 +3575,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>51.158999999999999</v>
       </c>
@@ -3606,7 +3601,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>26.515999999999998</v>
       </c>
@@ -3632,7 +3627,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>8.5090000000000003</v>
       </c>
@@ -3658,7 +3653,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="99" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>6.2E-2</v>
       </c>
@@ -3684,7 +3679,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="100" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>34.536000000000001</v>
       </c>
@@ -3710,7 +3705,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="101" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>47.003</v>
       </c>
@@ -3736,7 +3731,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="102" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>50.484000000000002</v>
       </c>
@@ -3762,7 +3757,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="103" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>58.701000000000001</v>
       </c>
@@ -3788,7 +3783,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="104" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>55.085999999999999</v>
       </c>
@@ -3814,7 +3809,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="105" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>46.152000000000001</v>
       </c>
@@ -3840,7 +3835,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="106" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>40.226999999999997</v>
       </c>
@@ -3866,7 +3861,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="107" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>35.857999999999997</v>
       </c>
@@ -3892,7 +3887,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="108" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>40.104999999999997</v>
       </c>
@@ -3918,7 +3913,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>20.521000000000001</v>
       </c>
@@ -3944,7 +3939,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="110" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>20</v>
       </c>
@@ -3970,7 +3965,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="111" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>1.976</v>
       </c>
@@ -3996,7 +3991,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="112" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>5.9850000000000003</v>
       </c>
@@ -4022,7 +4017,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="113" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>1.0780000000000001</v>
       </c>
@@ -4048,7 +4043,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="114" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>1.107</v>
       </c>
@@ -4074,7 +4069,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="115" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>14.271000000000001</v>
       </c>
@@ -4100,7 +4095,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="116" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>12.242000000000001</v>
       </c>
@@ -4126,7 +4121,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="117" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>10.08</v>
       </c>
@@ -4152,7 +4147,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="118" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>20</v>
       </c>
@@ -4178,7 +4173,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="119" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>28.8</v>
       </c>
@@ -4204,7 +4199,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="120" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>35.784520000000001</v>
       </c>
@@ -4230,7 +4225,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="121" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>58.820999999999998</v>
       </c>
@@ -4256,7 +4251,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="122" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>39.454999999999998</v>
       </c>
@@ -4282,7 +4277,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="123" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>30.347000000000001</v>
       </c>
@@ -4308,7 +4303,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="124" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>29.776</v>
       </c>
@@ -4334,7 +4329,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="125" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>28.7</v>
       </c>
@@ -4360,7 +4355,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="126" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>12.553000000000001</v>
       </c>
@@ -4386,7 +4381,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="127" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>9.3979999999999997</v>
       </c>
@@ -4412,7 +4407,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="128" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>19.957000000000001</v>
       </c>
@@ -4438,7 +4433,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="129" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>35.055</v>
       </c>
@@ -4464,7 +4459,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="130" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>46.591999999999999</v>
       </c>
@@ -4490,7 +4485,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="131" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>20.178000000000001</v>
       </c>
@@ -4516,7 +4511,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="132" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>27.425000000000001</v>
       </c>
@@ -4542,7 +4537,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="133" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>54.71</v>
       </c>
@@ -4568,7 +4563,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="134" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>42.854999999999997</v>
       </c>
@@ -4594,7 +4589,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="135" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>39.960999999999999</v>
       </c>
@@ -4620,7 +4615,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="136" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>12.052</v>
       </c>
@@ -4646,7 +4641,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="137" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>5.2469999999999999</v>
       </c>
@@ -4672,7 +4667,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="138" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>28.312000000000001</v>
       </c>
@@ -4698,7 +4693,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="139" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>40.366999999999997</v>
       </c>
@@ -4724,7 +4719,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="140" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>7.6239999999999997</v>
       </c>
@@ -4750,7 +4745,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="141" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>26.797000000000001</v>
       </c>
@@ -4776,7 +4771,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="142" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>46.545000000000002</v>
       </c>
@@ -4802,7 +4797,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="143" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>56.892000000000003</v>
       </c>
@@ -4828,7 +4823,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="144" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>39.091000000000001</v>
       </c>
@@ -4854,7 +4849,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="145" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>18.058</v>
       </c>
@@ -4880,7 +4875,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="146" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>11.662000000000001</v>
       </c>
@@ -4906,7 +4901,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="147" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>31.742999999999999</v>
       </c>
@@ -4932,7 +4927,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="148" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>54.612000000000002</v>
       </c>
@@ -4958,7 +4953,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="149" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>6.306</v>
       </c>
@@ -4984,7 +4979,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="150" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>13.823</v>
       </c>
@@ -5010,7 +5005,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="151" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>13.554</v>
       </c>
@@ -5036,7 +5031,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="152" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>19.936</v>
       </c>
@@ -5062,7 +5057,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="153" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>26.571999999999999</v>
       </c>
@@ -5088,7 +5083,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="154" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>27.271000000000001</v>
       </c>
@@ -5114,7 +5109,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="155" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>46.710999999999999</v>
       </c>
@@ -5140,7 +5135,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="156" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>49.423999999999999</v>
       </c>
@@ -5166,7 +5161,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="157" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>44.317999999999998</v>
       </c>
@@ -5192,7 +5187,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="158" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>54.41</v>
       </c>
@@ -5218,7 +5213,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="159" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>54.844999999999999</v>
       </c>
@@ -5244,7 +5239,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="160" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>40.728999999999999</v>
       </c>
@@ -5270,7 +5265,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="161" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>33.277000000000001</v>
       </c>
@@ -5296,7 +5291,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="162" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>24.088999999999999</v>
       </c>
@@ -5322,7 +5317,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="163" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>21.363</v>
       </c>
@@ -5348,7 +5343,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="164" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>16.138000000000002</v>
       </c>
@@ -5374,7 +5369,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="165" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>15.233000000000001</v>
       </c>
@@ -5400,7 +5395,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="166" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>5.4850000000000003</v>
       </c>
@@ -5426,7 +5421,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="167" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>3.82</v>
       </c>
@@ -5452,7 +5447,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="168" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>5.335</v>
       </c>
@@ -5478,7 +5473,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="169" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>13.994999999999999</v>
       </c>
@@ -5504,7 +5499,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="170" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>29.786999999999999</v>
       </c>
@@ -5530,7 +5525,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="171" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>21.72</v>
       </c>
@@ -5556,7 +5551,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="172" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>20</v>
       </c>
@@ -5582,7 +5577,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="173" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>58.034999999999997</v>
       </c>
@@ -5608,7 +5603,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="174" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>52.643000000000001</v>
       </c>
@@ -5634,7 +5629,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="175" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>54.502000000000002</v>
       </c>
@@ -5660,7 +5655,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="176" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>0.38300000000000001</v>
       </c>
@@ -5686,7 +5681,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="177" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>14.069000000000001</v>
       </c>
@@ -5712,7 +5707,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="178" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>16.603000000000002</v>
       </c>
@@ -5738,7 +5733,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="179" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>10.622</v>
       </c>
@@ -5764,7 +5759,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="180" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>20.928999999999998</v>
       </c>
@@ -5790,7 +5785,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="181" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>41.715000000000003</v>
       </c>
@@ -5816,7 +5811,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="182" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>40.06</v>
       </c>
@@ -5842,7 +5837,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="183" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>42.969000000000001</v>
       </c>
@@ -5868,7 +5863,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="184" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>47.084000000000003</v>
       </c>
@@ -5894,7 +5889,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="185" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>50.088000000000001</v>
       </c>
@@ -5920,7 +5915,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="186" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>51.237000000000002</v>
       </c>
@@ -5946,7 +5941,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="187" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>57.445999999999998</v>
       </c>
@@ -5972,7 +5967,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="188" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>56.848999999999997</v>
       </c>
@@ -5998,7 +5993,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="189" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>40.429000000000002</v>
       </c>
@@ -6024,7 +6019,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="190" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>57.16</v>
       </c>
@@ -6050,7 +6045,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="191" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>28.167999999999999</v>
       </c>
@@ -6076,7 +6071,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="192" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>33.124000000000002</v>
       </c>
@@ -6102,7 +6097,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="193" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>6.7859999999999996</v>
       </c>
@@ -6128,7 +6123,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="194" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>4.8739999999999997</v>
       </c>
@@ -6154,7 +6149,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="195" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>-0.13300000000000001</v>
       </c>
@@ -6180,7 +6175,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="196" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>5.7080000000000002</v>
       </c>
@@ -6206,7 +6201,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="197" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>10.397</v>
       </c>
@@ -6232,7 +6227,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="198" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>16.859000000000002</v>
       </c>
@@ -6258,7 +6253,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="199" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>19.312999999999999</v>
       </c>
@@ -6284,7 +6279,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="200" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A200">
         <v>17.513999999999999</v>
       </c>
@@ -6310,7 +6305,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="201" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>11.429</v>
       </c>
@@ -6336,7 +6331,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="202" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A202">
         <v>5.2210000000000001</v>
       </c>
@@ -6362,7 +6357,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="203" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A203">
         <v>33.582999999999998</v>
       </c>
@@ -6388,7 +6383,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="204" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A204">
         <v>32.387</v>
       </c>
@@ -6414,7 +6409,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="205" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A205">
         <v>48.116999999999997</v>
       </c>
@@ -6440,7 +6435,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="206" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A206">
         <v>40.945</v>
       </c>
@@ -6466,7 +6461,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="207" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A207">
         <v>40.365000000000002</v>
       </c>
@@ -6492,7 +6487,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="208" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A208">
         <v>18.260999999999999</v>
       </c>
@@ -6518,7 +6513,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="209" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A209">
         <v>37.796999999999997</v>
       </c>
@@ -6544,7 +6539,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="210" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A210">
         <v>6.6840000000000002</v>
       </c>
@@ -6570,7 +6565,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="211" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A211">
         <v>33.831000000000003</v>
       </c>
@@ -6596,7 +6591,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="212" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A212">
         <v>60.298999999999999</v>
       </c>
@@ -6622,7 +6617,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="213" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A213">
         <v>50.246000000000002</v>
       </c>
@@ -6648,7 +6643,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="214" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A214">
         <v>33.847000000000001</v>
       </c>
@@ -6674,7 +6669,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="215" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A215">
         <v>13.811999999999999</v>
       </c>
@@ -6700,7 +6695,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="216" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A216">
         <v>9.2940000000000005</v>
       </c>
@@ -6726,7 +6721,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="217" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A217">
         <v>29.492999999999999</v>
       </c>
@@ -6752,7 +6747,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="218" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A218">
         <v>50.076999999999998</v>
       </c>
@@ -6778,7 +6773,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A219">
         <v>41.985999999999997</v>
       </c>
@@ -6804,7 +6799,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A220">
         <v>57.16</v>
       </c>
@@ -6830,7 +6825,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="221" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A221">
         <v>48.2</v>
       </c>
@@ -6856,7 +6851,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="222" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A222">
         <v>44.115000000000002</v>
       </c>
@@ -6882,7 +6877,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A223">
         <v>45.84</v>
       </c>
@@ -6908,7 +6903,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="224" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A224">
         <v>46.207000000000001</v>
       </c>
@@ -6934,7 +6929,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="225" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A225">
         <v>39.526000000000003</v>
       </c>
@@ -6960,7 +6955,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="226" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A226">
         <v>24.196000000000002</v>
       </c>
@@ -6986,7 +6981,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="227" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A227">
         <v>20.218</v>
       </c>
@@ -7012,7 +7007,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="228" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A228">
         <v>25.507000000000001</v>
       </c>
@@ -7038,7 +7033,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="229" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A229">
         <v>19.843</v>
       </c>
@@ -7064,7 +7059,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="230" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A230">
         <v>27.556000000000001</v>
       </c>
@@ -7090,7 +7085,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="231" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A231">
         <v>11.571</v>
       </c>
@@ -7116,7 +7111,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="232" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A232">
         <v>2.67</v>
       </c>
@@ -7142,7 +7137,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="233" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A233">
         <v>9.6679999999999993</v>
       </c>
@@ -7168,7 +7163,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="234" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A234">
         <v>7.1529999999999996</v>
       </c>
@@ -7194,7 +7189,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="235" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A235">
         <v>17.147919999999999</v>
       </c>
@@ -7220,7 +7215,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="236" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A236">
         <v>17.672999999999998</v>
       </c>
@@ -7246,7 +7241,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="237" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A237">
         <v>2.0670000000000002</v>
       </c>
@@ -7272,7 +7267,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="238" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A238">
         <v>4.3639999999999999</v>
       </c>
@@ -7298,7 +7293,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="239" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A239">
         <v>13.106999999999999</v>
       </c>
@@ -7324,7 +7319,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="240" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A240">
         <v>29.492000000000001</v>
       </c>
@@ -7350,7 +7345,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="241" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A241">
         <v>34.116999999999997</v>
       </c>
@@ -7376,7 +7371,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="242" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A242">
         <v>32.079000000000001</v>
       </c>
@@ -7402,7 +7397,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="243" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A243">
         <v>54.86</v>
       </c>
@@ -7428,7 +7423,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="244" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A244">
         <v>52.305999999999997</v>
       </c>
@@ -7454,7 +7449,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="245" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A245">
         <v>54.301000000000002</v>
       </c>
@@ -7480,7 +7475,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="246" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A246">
         <v>32.432000000000002</v>
       </c>
@@ -7506,7 +7501,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="247" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A247">
         <v>35.1050325</v>
       </c>
@@ -7532,7 +7527,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="248" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A248">
         <v>46.171999999999997</v>
       </c>
@@ -7558,7 +7553,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="249" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A249">
         <v>45.009</v>
       </c>
@@ -7584,7 +7579,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="250" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A250">
         <v>57.304000000000002</v>
       </c>
@@ -7610,7 +7605,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="251" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A251">
         <v>59.360999999999997</v>
       </c>
@@ -7636,7 +7631,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="252" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A252">
         <v>42.912999999999997</v>
       </c>
@@ -7662,7 +7657,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="253" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A253">
         <v>45.084000000000003</v>
       </c>
@@ -7688,7 +7683,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="254" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A254">
         <v>57.274000000000001</v>
       </c>
@@ -7714,7 +7709,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="255" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A255">
         <v>36.075000000000003</v>
       </c>
@@ -7740,7 +7735,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="256" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A256">
         <v>9.157</v>
       </c>
@@ -7766,7 +7761,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="257" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A257">
         <v>9.8070000000000004</v>
       </c>
@@ -7792,7 +7787,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="258" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A258">
         <v>17.795000000000002</v>
       </c>
@@ -7818,7 +7813,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="259" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A259">
         <v>17.324000000000002</v>
       </c>
@@ -7844,7 +7839,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="260" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A260">
         <v>4.2370000000000001</v>
       </c>
@@ -7870,7 +7865,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="261" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A261">
         <v>4.5919999999999996</v>
       </c>
@@ -7896,7 +7891,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="262" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A262">
         <v>6.327</v>
       </c>
@@ -7922,7 +7917,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="263" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A263">
         <v>6.3929999999999998</v>
       </c>
@@ -7948,7 +7943,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="264" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A264">
         <v>16.254000000000001</v>
       </c>
@@ -7974,7 +7969,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="265" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A265">
         <v>7.16</v>
       </c>
@@ -8000,7 +7995,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="266" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A266">
         <v>27.161999999999999</v>
       </c>
@@ -8026,7 +8021,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="267" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A267">
         <v>30.991</v>
       </c>
@@ -8052,7 +8047,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="268" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A268">
         <v>30.561</v>
       </c>
@@ -8078,7 +8073,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="269" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A269">
         <v>35.802999999999997</v>
       </c>
@@ -8104,7 +8099,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="270" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A270">
         <v>46.997999999999998</v>
       </c>
@@ -8130,7 +8125,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="271" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A271">
         <v>53.887999999999998</v>
       </c>
@@ -8156,7 +8151,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="272" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A272">
         <v>52.084000000000003</v>
       </c>
@@ -8182,7 +8177,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="273" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A273">
         <v>43.781999999999996</v>
       </c>
@@ -8208,7 +8203,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="274" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A274">
         <v>39.909999999999997</v>
       </c>
@@ -8234,7 +8229,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="275" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A275">
         <v>4.194</v>
       </c>
@@ -8260,7 +8255,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="276" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A276">
         <v>33.485999999999997</v>
       </c>
@@ -8286,7 +8281,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="277" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A277">
         <v>47.706000000000003</v>
       </c>
@@ -8312,7 +8307,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="278" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A278">
         <v>57.844000000000001</v>
       </c>
@@ -8338,7 +8333,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="279" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A279">
         <v>39.436999999999998</v>
       </c>
@@ -8364,7 +8359,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="280" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A280">
         <v>12.542</v>
       </c>
@@ -8390,7 +8385,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="281" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A281">
         <v>3.468</v>
       </c>
@@ -8416,7 +8411,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="282" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A282">
         <v>36.06</v>
       </c>
@@ -8442,7 +8437,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="283" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A283">
         <v>58.261000000000003</v>
       </c>
@@ -8468,7 +8463,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="284" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A284">
         <v>41.548999999999999</v>
       </c>
@@ -8494,7 +8489,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="285" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A285">
         <v>23.501999999999999</v>
       </c>
@@ -8520,7 +8515,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="286" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A286">
         <v>1.1120000000000001</v>
       </c>
@@ -8546,7 +8541,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="287" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A287">
         <v>14.839</v>
       </c>
@@ -8572,7 +8567,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="288" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A288">
         <v>40.770000000000003</v>
       </c>
@@ -8598,7 +8593,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="289" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A289">
         <v>37.048000000000002</v>
       </c>
@@ -8624,7 +8619,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="290" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A290">
         <v>55.906999999999996</v>
       </c>
@@ -8650,7 +8645,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="291" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A291">
         <v>28.015000000000001</v>
       </c>
@@ -8676,7 +8671,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="292" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A292">
         <v>18.012</v>
       </c>
@@ -8702,7 +8697,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="293" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A293">
         <v>0.65</v>
       </c>
@@ -8728,7 +8723,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="294" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A294">
         <v>40</v>
       </c>
@@ -8754,7 +8749,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="295" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A295">
         <v>55.521000000000001</v>
       </c>
@@ -8780,7 +8775,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="296" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A296">
         <v>40.383000000000003</v>
       </c>
@@ -8806,7 +8801,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="297" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A297">
         <v>28.77</v>
       </c>
@@ -8832,7 +8827,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="298" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A298">
         <v>8.9649999999999999</v>
       </c>
@@ -8858,7 +8853,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="299" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A299">
         <v>9.8699999999999992</v>
       </c>
@@ -8884,7 +8879,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="300" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A300">
         <v>21.207000000000001</v>
       </c>
@@ -8910,7 +8905,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="301" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A301">
         <v>50.981999999999999</v>
       </c>
@@ -8936,7 +8931,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="302" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A302">
         <v>35.92</v>
       </c>
@@ -8962,7 +8957,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="303" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A303">
         <v>41.34</v>
       </c>
@@ -8988,7 +8983,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="304" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A304">
         <v>45.88</v>
       </c>
@@ -9014,7 +9009,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="305" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A305">
         <v>52.41</v>
       </c>
@@ -9040,7 +9035,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="306" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A306">
         <v>55.32</v>
       </c>
@@ -9066,7 +9061,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="307" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A307">
         <v>49.73</v>
       </c>
@@ -9092,7 +9087,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="308" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A308">
         <v>50.86</v>
       </c>
@@ -9118,7 +9113,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="309" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A309">
         <v>53.9</v>
       </c>
@@ -9144,7 +9139,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="310" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A310">
         <v>57.61</v>
       </c>
@@ -9171,13 +9166,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="H1:H310" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Cplot13"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="H1:H310" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Update: addition of 3D microhabitat analyses
</commit_message>
<xml_diff>
--- a/Data/sensor_locations_all_plots.xlsx
+++ b/Data/sensor_locations_all_plots.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ugentbe-my.sharepoint.com/personal/egvdwall_vandewalle_ugent_be/Documents/Documenten/PhD CAVElab/Code PhD/ForEdgeClimOnPanama/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{1F05EFE1-A1B1-46D8-97A0-A405852F5B9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D00FA1E-6A1B-410F-B607-17E12D30D81A}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{1F05EFE1-A1B1-46D8-97A0-A405852F5B9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B3AFC55-4CF6-4B16-9AEF-97D6CC7190A1}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sensor_locations" sheetId="1" r:id="rId1"/>
@@ -3502,7 +3502,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>5.8650000000000002</v>
       </c>
@@ -3528,7 +3528,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>39.704999999999998</v>
       </c>
@@ -3554,7 +3554,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>51.826999999999998</v>
       </c>
@@ -3580,7 +3580,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>51.158999999999999</v>
       </c>
@@ -3606,7 +3606,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>26.515999999999998</v>
       </c>
@@ -3632,7 +3632,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>8.5090000000000003</v>
       </c>
@@ -3658,7 +3658,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="99" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>6.2E-2</v>
       </c>
@@ -3684,7 +3684,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="100" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>34.536000000000001</v>
       </c>
@@ -3710,7 +3710,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="101" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>47.003</v>
       </c>
@@ -3736,7 +3736,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="102" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>50.484000000000002</v>
       </c>
@@ -3762,7 +3762,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="103" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>58.701000000000001</v>
       </c>
@@ -3788,7 +3788,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="104" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>55.085999999999999</v>
       </c>
@@ -3814,7 +3814,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="105" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>46.152000000000001</v>
       </c>
@@ -3840,7 +3840,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="106" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>40.226999999999997</v>
       </c>
@@ -3866,7 +3866,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="107" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>35.857999999999997</v>
       </c>
@@ -3892,7 +3892,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="108" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>40.104999999999997</v>
       </c>
@@ -3918,7 +3918,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>20.521000000000001</v>
       </c>
@@ -3944,7 +3944,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="110" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>20</v>
       </c>
@@ -3970,7 +3970,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="111" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>1.976</v>
       </c>
@@ -3996,7 +3996,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="112" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>5.9850000000000003</v>
       </c>
@@ -4022,7 +4022,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="113" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>1.0780000000000001</v>
       </c>
@@ -4048,7 +4048,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="114" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>1.107</v>
       </c>
@@ -4074,7 +4074,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="115" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>14.271000000000001</v>
       </c>
@@ -4100,7 +4100,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="116" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>12.242000000000001</v>
       </c>
@@ -4126,7 +4126,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="117" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>10.08</v>
       </c>
@@ -4152,7 +4152,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="118" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>20</v>
       </c>
@@ -4178,7 +4178,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="119" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>28.8</v>
       </c>
@@ -4204,7 +4204,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="120" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>35.784520000000001</v>
       </c>
@@ -4230,7 +4230,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="121" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>58.820999999999998</v>
       </c>
@@ -4256,7 +4256,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="122" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>39.454999999999998</v>
       </c>
@@ -4282,7 +4282,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="123" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>30.347000000000001</v>
       </c>
@@ -4308,7 +4308,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="124" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>29.776</v>
       </c>
@@ -4334,7 +4334,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="125" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>28.7</v>
       </c>
@@ -4360,7 +4360,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="126" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>12.553000000000001</v>
       </c>
@@ -4386,7 +4386,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="127" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>9.3979999999999997</v>
       </c>
@@ -4412,7 +4412,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="128" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>19.957000000000001</v>
       </c>
@@ -4438,7 +4438,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="129" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>35.055</v>
       </c>
@@ -4464,7 +4464,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="130" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>46.591999999999999</v>
       </c>
@@ -8702,7 +8702,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="293" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A293">
         <v>0.65</v>
       </c>
@@ -8728,7 +8728,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="294" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A294">
         <v>40</v>
       </c>
@@ -8754,7 +8754,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="295" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A295">
         <v>55.521000000000001</v>
       </c>
@@ -8780,7 +8780,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="296" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A296">
         <v>40.383000000000003</v>
       </c>
@@ -8806,7 +8806,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="297" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A297">
         <v>28.77</v>
       </c>
@@ -8832,7 +8832,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="298" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A298">
         <v>8.9649999999999999</v>
       </c>
@@ -8858,7 +8858,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="299" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A299">
         <v>9.8699999999999992</v>
       </c>
@@ -8884,7 +8884,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="300" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A300">
         <v>21.207000000000001</v>
       </c>
@@ -8910,7 +8910,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="301" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A301">
         <v>50.981999999999999</v>
       </c>
@@ -9066,7 +9066,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="307" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A307">
         <v>49.73</v>
       </c>
@@ -9092,7 +9092,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="308" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A308">
         <v>50.86</v>
       </c>
@@ -9118,7 +9118,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="309" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A309">
         <v>53.9</v>
       </c>
@@ -9144,7 +9144,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="310" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A310">
         <v>57.61</v>
       </c>
@@ -9174,7 +9174,7 @@
   <autoFilter ref="H1:H310" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="0">
       <filters>
-        <filter val="Cplot16"/>
+        <filter val="Cplot08"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>